<commit_message>
Add library signage HTML template and unit tests for API constants
- Created an HTML file for printing library signage in A4 landscape format, including sections for various departments with QR codes.
- Added unit tests for the `bookByAccession` method in `api_constants_test.dart` to ensure correct URL generation and handling of special characters.
</commit_message>
<xml_diff>
--- a/backend/data/Datasource.xlsx
+++ b/backend/data/Datasource.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jimmy\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C401457-EBDF-4141-AAE8-7C219A2BC51B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE033920-3BA4-459C-8B2F-27A5FF3DEE0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
     <sheet name="articles" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">books!$A$1:$N$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">books!$A$1:$O$51</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2077" uniqueCount="1575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2128" uniqueCount="1625">
   <si>
     <t>BibID</t>
   </si>
@@ -4762,13 +4762,163 @@
   </si>
   <si>
     <t>10.1146/annurev-fluid-122414-034353</t>
+  </si>
+  <si>
+    <t>الرقم العام</t>
+  </si>
+  <si>
+    <t>86</t>
+  </si>
+  <si>
+    <t>773</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>1040</t>
+  </si>
+  <si>
+    <t>413</t>
+  </si>
+  <si>
+    <t>1038</t>
+  </si>
+  <si>
+    <t>566</t>
+  </si>
+  <si>
+    <t>1282</t>
+  </si>
+  <si>
+    <t>1285</t>
+  </si>
+  <si>
+    <t>533</t>
+  </si>
+  <si>
+    <t>1019</t>
+  </si>
+  <si>
+    <t>697</t>
+  </si>
+  <si>
+    <t>588</t>
+  </si>
+  <si>
+    <t>441</t>
+  </si>
+  <si>
+    <t>167</t>
+  </si>
+  <si>
+    <t>330</t>
+  </si>
+  <si>
+    <t>175</t>
+  </si>
+  <si>
+    <t>729</t>
+  </si>
+  <si>
+    <t>368</t>
+  </si>
+  <si>
+    <t>1879</t>
+  </si>
+  <si>
+    <t>677</t>
+  </si>
+  <si>
+    <t>731</t>
+  </si>
+  <si>
+    <t>1467</t>
+  </si>
+  <si>
+    <t>1515</t>
+  </si>
+  <si>
+    <t>1415</t>
+  </si>
+  <si>
+    <t>1345</t>
+  </si>
+  <si>
+    <t>407</t>
+  </si>
+  <si>
+    <t>446</t>
+  </si>
+  <si>
+    <t>1207</t>
+  </si>
+  <si>
+    <t>293</t>
+  </si>
+  <si>
+    <t>1202</t>
+  </si>
+  <si>
+    <t>1353</t>
+  </si>
+  <si>
+    <t>1180</t>
+  </si>
+  <si>
+    <t>444</t>
+  </si>
+  <si>
+    <t>379</t>
+  </si>
+  <si>
+    <t>1182</t>
+  </si>
+  <si>
+    <t>1139</t>
+  </si>
+  <si>
+    <t>360</t>
+  </si>
+  <si>
+    <t>581</t>
+  </si>
+  <si>
+    <t>968</t>
+  </si>
+  <si>
+    <t>548</t>
+  </si>
+  <si>
+    <t>1445</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>346</t>
+  </si>
+  <si>
+    <t>285</t>
+  </si>
+  <si>
+    <t>1270</t>
+  </si>
+  <si>
+    <t>189</t>
+  </si>
+  <si>
+    <t>198</t>
+  </si>
+  <si>
+    <t>Null</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -4812,8 +4962,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4843,6 +5003,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -4853,11 +5025,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -4884,12 +5057,63 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{755676BB-AC15-4461-8DAA-00BB870CD54C}"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -5256,2279 +5480,2436 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="82.36328125" customWidth="1"/>
-    <col min="4" max="4" width="17.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.08984375" customWidth="1"/>
-    <col min="12" max="12" width="27" customWidth="1"/>
-    <col min="13" max="14" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.36328125" style="22" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" style="30" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" customWidth="1"/>
+    <col min="4" max="4" width="82.36328125" customWidth="1"/>
+    <col min="5" max="5" width="17.1796875" customWidth="1"/>
+    <col min="6" max="6" width="6.1796875" customWidth="1"/>
+    <col min="7" max="7" width="25.7265625" customWidth="1"/>
+    <col min="8" max="8" width="8.6328125" customWidth="1"/>
+    <col min="9" max="9" width="10.90625" customWidth="1"/>
+    <col min="10" max="10" width="16.6328125" customWidth="1"/>
+    <col min="11" max="11" width="21" customWidth="1"/>
+    <col min="12" max="12" width="19.08984375" customWidth="1"/>
+    <col min="13" max="13" width="27" customWidth="1"/>
+    <col min="14" max="15" width="18.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="26" t="s">
+        <v>1575</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="28" t="s">
+        <v>1600</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G2" s="2">
+      <c r="H2" s="2">
         <v>2003</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="K2" s="4">
+      <c r="L2" s="4">
         <v>31</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="O2" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="28" t="s">
+        <v>1601</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="2">
+      <c r="H3" s="2">
         <v>2010</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="4">
+      <c r="L3" s="4">
         <v>33</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="M3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="N3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="O3" s="5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2">
+    <row r="4" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="3">
         <v>13017812</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="28" t="s">
+        <v>1599</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="2">
+      <c r="H4" s="2">
         <v>2019</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K4" s="4">
+      <c r="L4" s="4">
         <v>31</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="M4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N4" s="5" t="s">
+      <c r="O4" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="28" t="s">
+        <v>1602</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="G5" s="2">
+      <c r="H5" s="2">
         <v>2003</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="K5" s="2">
+      <c r="L5" s="2">
         <v>33</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="M5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="N5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N5" s="5" t="s">
+      <c r="O5" s="5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="28" t="s">
+        <v>1603</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>356</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="G6" s="2">
+      <c r="H6" s="2">
         <v>2002</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>360</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>357</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="K6" s="2" t="s">
         <v>361</v>
       </c>
-      <c r="K6" s="2">
+      <c r="L6" s="2">
         <v>37</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="M6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M6" s="2" t="s">
+      <c r="N6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N6" s="5" t="s">
+      <c r="O6" s="5" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="7" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="25" t="s">
         <v>363</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="28" t="s">
+        <v>1615</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="I7" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="J7" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
         <v>370</v>
       </c>
-      <c r="K7" s="2">
+      <c r="L7" s="2">
         <v>39</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="M7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="N7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="O7" s="5" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="8" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="28" t="s">
+        <v>1604</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G8" s="2">
+      <c r="H8" s="2">
         <v>2007</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="I8" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="J8" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="K8" s="2">
+      <c r="L8" s="2">
         <v>39</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="M8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="N8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N8" s="5" t="s">
+      <c r="O8" s="5" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
         <v>372</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="28" t="s">
+        <v>1605</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="J9" s="6" t="s">
         <v>374</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="K9" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="K9" s="2">
+      <c r="L9" s="2">
         <v>34</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="M9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="N9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N9" s="5" t="s">
+      <c r="O9" s="5" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="10" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="28" t="s">
+        <v>1606</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="G10" s="2">
+      <c r="H10" s="2">
         <v>2002</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="I10" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="I10" s="3">
+      <c r="J10" s="3">
         <v>521781752</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="K10" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="K10" s="2">
+      <c r="L10" s="2">
         <v>38</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="M10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="N10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N10" s="5" t="s">
+      <c r="O10" s="5" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="28" t="s">
+        <v>1607</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="G11" s="2">
+      <c r="H11" s="2">
         <v>2008</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="I11" s="3">
+      <c r="J11" s="3">
         <v>9788123915791</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="K11" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="K11" s="2">
+      <c r="L11" s="2">
         <v>33</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="M11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M11" s="2" t="s">
+      <c r="N11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N11" s="5" t="s">
+      <c r="O11" s="5" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="12" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
+    <row r="12" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="10" t="s">
         <v>380</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="29" t="s">
+        <v>1583</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>381</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D12" s="7" t="s">
         <v>384</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="E12" s="7" t="s">
         <v>383</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="F12" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="G12" s="7" t="s">
         <v>385</v>
       </c>
-      <c r="G12" s="7">
+      <c r="H12" s="7">
         <v>2016</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="I12" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="J12" s="7" t="s">
         <v>382</v>
       </c>
-      <c r="J12" s="7" t="s">
+      <c r="K12" s="7" t="s">
         <v>386</v>
       </c>
-      <c r="K12" s="7">
+      <c r="L12" s="7">
         <v>64</v>
       </c>
-      <c r="L12" s="8" t="s">
+      <c r="M12" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="M12" s="8" t="s">
+      <c r="N12" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="N12" s="9" t="s">
+      <c r="O12" s="9" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="13" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="7" t="s">
+    <row r="13" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="29" t="s">
+        <v>1584</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="E13" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="F13" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="G13" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G13" s="7">
+      <c r="H13" s="7">
         <v>2010</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="I13" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="J13" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="J13" s="7" t="s">
+      <c r="K13" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="K13" s="7">
+      <c r="L13" s="7">
         <v>66</v>
       </c>
-      <c r="L13" s="8" t="s">
+      <c r="M13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="M13" s="8" t="s">
+      <c r="N13" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="N13" s="9" t="s">
+      <c r="O13" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="7" t="s">
+    <row r="14" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="29" t="s">
+        <v>1616</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="D14" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="E14" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="F14" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="G14" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G14" s="7">
+      <c r="H14" s="7">
         <v>2006</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="I14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I14" s="10" t="s">
+      <c r="J14" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="J14" s="7" t="s">
+      <c r="K14" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="K14" s="7">
+      <c r="L14" s="7">
         <v>62</v>
       </c>
-      <c r="L14" s="8" t="s">
+      <c r="M14" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="M14" s="7" t="s">
+      <c r="N14" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N14" s="9" t="s">
+      <c r="O14" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="7" t="s">
+    <row r="15" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="10" t="s">
         <v>388</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="29" t="s">
+        <v>1585</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>389</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="D15" s="7" t="s">
         <v>391</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="E15" s="7" t="s">
         <v>390</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="F15" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="G15" s="7" t="s">
         <v>392</v>
       </c>
-      <c r="G15" s="7">
+      <c r="H15" s="7">
         <v>2016</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="I15" s="7" t="s">
         <v>393</v>
       </c>
-      <c r="I15" s="7">
+      <c r="J15" s="7">
         <v>9780415746281</v>
       </c>
-      <c r="J15" s="7" t="s">
+      <c r="K15" s="7" t="s">
         <v>394</v>
       </c>
-      <c r="K15" s="7">
+      <c r="L15" s="7">
         <v>62</v>
       </c>
-      <c r="L15" s="8" t="s">
+      <c r="M15" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="M15" s="7" t="s">
+      <c r="N15" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N15" s="9" t="s">
+      <c r="O15" s="9" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="16" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="7" t="s">
+    <row r="16" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="29" t="s">
+        <v>1586</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="D16" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="F16" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="G16" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="G16" s="7">
+      <c r="H16" s="7">
         <v>2008</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="I16" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="I16" s="10">
+      <c r="J16" s="10">
         <v>9788957702130</v>
       </c>
-      <c r="J16" s="7" t="s">
+      <c r="K16" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="K16" s="7">
+      <c r="L16" s="7">
         <v>67</v>
       </c>
-      <c r="L16" s="8" t="s">
+      <c r="M16" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="M16" s="7" t="s">
+      <c r="N16" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="N16" s="7" t="s">
+      <c r="O16" s="7" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="17" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="7" t="s">
+    <row r="17" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="29" t="s">
+        <v>1587</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="D17" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="E17" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="F17" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="G17" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="G17" s="7">
+      <c r="H17" s="7">
         <v>2007</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="I17" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="I17" s="10">
+      <c r="J17" s="10">
         <v>8957701591</v>
       </c>
-      <c r="J17" s="7" t="s">
+      <c r="K17" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="K17" s="7">
+      <c r="L17" s="7">
         <v>68</v>
       </c>
-      <c r="L17" s="8" t="s">
+      <c r="M17" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="M17" s="7" t="s">
+      <c r="N17" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N17" s="7" t="s">
+      <c r="O17" s="7" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="18" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="7" t="s">
+    <row r="18" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="10" t="s">
         <v>396</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="29" t="s">
+        <v>1588</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D18" s="7" t="s">
         <v>398</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="E18" s="7" t="s">
         <v>403</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="F18" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="G18" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="G18" s="7">
+      <c r="H18" s="7">
         <v>2009</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="I18" s="7" t="s">
         <v>400</v>
       </c>
-      <c r="I18" s="7">
+      <c r="J18" s="7">
         <v>9781844077717</v>
       </c>
-      <c r="J18" s="7" t="s">
+      <c r="K18" s="7" t="s">
         <v>401</v>
       </c>
-      <c r="K18" s="7">
+      <c r="L18" s="7">
         <v>64</v>
       </c>
-      <c r="L18" s="8" t="s">
+      <c r="M18" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="M18" s="7" t="s">
+      <c r="N18" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N18" s="9" t="s">
+      <c r="O18" s="9" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="19" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="7" t="s">
+    <row r="19" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="10" t="s">
         <v>404</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="29" t="s">
+        <v>1589</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>405</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="E19" s="7" t="s">
         <v>407</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="F19" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="G19" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="G19" s="7">
+      <c r="H19" s="7">
         <v>2001</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="I19" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="I19" s="11" t="s">
+      <c r="J19" s="11" t="s">
         <v>406</v>
       </c>
-      <c r="J19" s="7" t="s">
+      <c r="K19" s="7" t="s">
         <v>409</v>
       </c>
-      <c r="K19" s="7">
+      <c r="L19" s="7">
         <v>64</v>
       </c>
-      <c r="L19" s="8" t="s">
+      <c r="M19" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="M19" s="7" t="s">
+      <c r="N19" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N19" s="9" t="s">
+      <c r="O19" s="9" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="20" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="7" t="s">
+    <row r="20" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="10" t="s">
         <v>411</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="29" t="s">
+        <v>1590</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>412</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="D20" s="7" t="s">
         <v>414</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="E20" s="7" t="s">
         <v>413</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="F20" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="G20" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="G20" s="7">
+      <c r="H20" s="7">
         <v>1999</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="I20" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="I20" s="12" t="s">
+      <c r="J20" s="12" t="s">
         <v>416</v>
       </c>
-      <c r="J20" s="7" t="s">
+      <c r="K20" s="7" t="s">
         <v>415</v>
       </c>
-      <c r="K20" s="7">
+      <c r="L20" s="7">
         <v>64</v>
       </c>
-      <c r="L20" s="8" t="s">
+      <c r="M20" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="M20" s="7" t="s">
+      <c r="N20" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N20" s="9" t="s">
+      <c r="O20" s="9" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="21" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="7" t="s">
+    <row r="21" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="25" t="s">
         <v>120</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="29" t="s">
+        <v>1617</v>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="D21" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="E21" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="F21" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="G21" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G21" s="7">
+      <c r="H21" s="7">
         <v>2015</v>
       </c>
-      <c r="H21" s="7" t="s">
+      <c r="I21" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="I21" s="10">
+      <c r="J21" s="10">
         <v>9788957705582</v>
       </c>
-      <c r="J21" s="7" t="s">
+      <c r="K21" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="K21" s="7">
+      <c r="L21" s="7">
         <v>62</v>
       </c>
-      <c r="L21" s="8" t="s">
+      <c r="M21" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="M21" s="7" t="s">
+      <c r="N21" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N21" s="7" t="s">
+      <c r="O21" s="7" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="22" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="27" t="s">
+        <v>1609</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="F22" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G22" s="2">
+      <c r="H22" s="2">
         <v>1999</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="I22" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I22" s="3">
+      <c r="J22" s="3">
         <v>9772820595</v>
       </c>
-      <c r="J22" s="2" t="s">
+      <c r="K22" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="K22" s="2">
+      <c r="L22" s="2">
         <v>53</v>
       </c>
-      <c r="L22" s="4" t="s">
+      <c r="M22" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="M22" s="4" t="s">
+      <c r="N22" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="N22" s="2" t="s">
+      <c r="O22" s="2" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="23" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="27" t="s">
+        <v>1610</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G23" s="2">
+      <c r="H23" s="2">
         <v>2003</v>
       </c>
-      <c r="H23" s="2" t="s">
+      <c r="I23" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I23" s="3">
+      <c r="J23" s="3">
         <v>8121903483</v>
       </c>
-      <c r="J23" s="2" t="s">
+      <c r="K23" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="K23" s="2">
+      <c r="L23" s="2">
         <v>47</v>
       </c>
-      <c r="L23" s="4" t="s">
+      <c r="M23" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="M23" s="2" t="s">
+      <c r="N23" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N23" s="2" t="s">
+      <c r="O23" s="2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="24" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
+    <row r="24" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="27" t="s">
+        <v>1611</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="E24" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="G24" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="G24" s="2">
+      <c r="H24" s="2">
         <v>1990</v>
       </c>
-      <c r="H24" s="2" t="s">
+      <c r="I24" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="I24" s="3">
+      <c r="J24" s="3">
         <v>434904686</v>
       </c>
-      <c r="J24" s="2" t="s">
+      <c r="K24" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="K24" s="2">
+      <c r="L24" s="2">
         <v>44</v>
       </c>
-      <c r="L24" s="4" t="s">
+      <c r="M24" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="M24" s="2" t="s">
+      <c r="N24" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N24" s="2" t="s">
+      <c r="O24" s="2" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="25" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
+    <row r="25" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="25" t="s">
         <v>150</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="27" t="s">
+        <v>1618</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="D25" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="E25" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="F25" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="G25" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="G25" s="2">
+      <c r="H25" s="2">
         <v>1988</v>
       </c>
-      <c r="H25" s="2" t="s">
+      <c r="I25" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="I25" s="3">
+      <c r="J25" s="3">
         <v>841214379</v>
       </c>
-      <c r="J25" s="2" t="s">
+      <c r="K25" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="K25" s="2">
+      <c r="L25" s="2">
         <v>50</v>
       </c>
-      <c r="L25" s="4" t="s">
+      <c r="M25" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="M25" s="2" t="s">
+      <c r="N25" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N25" s="2" t="s">
+      <c r="O25" s="2" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="26" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
+    <row r="26" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="27" t="s">
+        <v>1612</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>331</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="E26" s="13" t="s">
         <v>335</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="G26" s="2">
+      <c r="H26" s="2">
         <v>2006</v>
       </c>
-      <c r="H26" s="2" t="s">
+      <c r="I26" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I26" s="6" t="s">
+      <c r="J26" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="J26" s="2" t="s">
+      <c r="K26" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="K26" s="2">
+      <c r="L26" s="2">
         <v>59</v>
       </c>
-      <c r="L26" s="4" t="s">
+      <c r="M26" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="M26" s="2" t="s">
+      <c r="N26" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N26" s="5" t="s">
+      <c r="O26" s="5" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="27" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="2" t="s">
+    <row r="27" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="27" t="s">
+        <v>1619</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="E27" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="F27" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="G27" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="G27" s="2">
+      <c r="H27" s="2">
         <v>1998</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="I27" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="I27" s="3">
+      <c r="J27" s="3">
         <v>333732014</v>
       </c>
-      <c r="J27" s="2" t="s">
+      <c r="K27" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="K27" s="2">
+      <c r="L27" s="2">
         <v>58</v>
       </c>
-      <c r="L27" s="4" t="s">
+      <c r="M27" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="M27" s="2" t="s">
+      <c r="N27" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N27" s="2" t="s">
+      <c r="O27" s="2" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="28" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="2" t="s">
+    <row r="28" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="27" t="s">
+        <v>1613</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="D28" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="E28" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="F28" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="G28" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="G28" s="2">
+      <c r="H28" s="2">
         <v>1998</v>
       </c>
-      <c r="H28" s="2" t="s">
+      <c r="I28" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="I28" s="3">
+      <c r="J28" s="3">
         <v>71153632</v>
       </c>
-      <c r="J28" s="2" t="s">
+      <c r="K28" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="K28" s="2">
+      <c r="L28" s="2">
         <v>46</v>
       </c>
-      <c r="L28" s="4" t="s">
+      <c r="M28" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="M28" s="2" t="s">
+      <c r="N28" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N28" s="2" t="s">
+      <c r="O28" s="2" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="29" spans="1:14" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="2">
+    <row r="29" spans="1:15" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="3">
         <v>11149220</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="27" t="s">
+        <v>1608</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>339</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="D29" s="14" t="s">
         <v>338</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="E29" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="F29" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="G29" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="G29" s="2">
+      <c r="H29" s="2">
         <v>2009</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="I29" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="I29" s="3" t="s">
+      <c r="J29" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="K29" s="2">
+      <c r="L29" s="2">
         <v>57</v>
       </c>
-      <c r="L29" s="4" t="s">
+      <c r="M29" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="M29" s="2" t="s">
+      <c r="N29" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N29" s="5" t="s">
+      <c r="O29" s="5" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="30" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
+    <row r="30" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="25" t="s">
         <v>184</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="27" t="s">
+        <v>1620</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="D30" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="E30" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="F30" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="G30" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="G30" s="2">
+      <c r="H30" s="2">
         <v>2000</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="I30" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I30" s="15" t="s">
+      <c r="J30" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="J30" s="2" t="s">
+      <c r="K30" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="K30" s="2">
+      <c r="L30" s="2">
         <v>45</v>
       </c>
-      <c r="L30" s="4" t="s">
+      <c r="M30" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="M30" s="2" t="s">
+      <c r="N30" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N30" s="2" t="s">
+      <c r="O30" s="2" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="31" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
+    <row r="31" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="27" t="s">
+        <v>1614</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="D31" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="E31" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="F31" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="G31" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="G31" s="2">
+      <c r="H31" s="2">
         <v>2003</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="I31" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="I31" s="16" t="s">
+      <c r="J31" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="J31" s="2" t="s">
+      <c r="K31" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="K31" s="2">
+      <c r="L31" s="2">
         <v>47</v>
       </c>
-      <c r="L31" s="4" t="s">
+      <c r="M31" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="M31" s="2" t="s">
+      <c r="N31" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N31" s="2" t="s">
+      <c r="O31" s="2" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="32" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="7">
+    <row r="32" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="10">
         <v>68143</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="29" t="s">
+        <v>1576</v>
+      </c>
+      <c r="C32" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="D32" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="E32" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="E32" s="8" t="s">
+      <c r="F32" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="G32" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="G32" s="7">
+      <c r="H32" s="7">
         <v>2000</v>
       </c>
-      <c r="H32" s="7" t="s">
+      <c r="I32" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="I32" s="10">
+      <c r="J32" s="10">
         <v>9770308374</v>
       </c>
-      <c r="J32" s="7" t="s">
+      <c r="K32" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="K32" s="7">
+      <c r="L32" s="7">
         <v>59</v>
       </c>
-      <c r="L32" s="8" t="s">
+      <c r="M32" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="M32" s="8" t="s">
+      <c r="N32" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="N32" s="7" t="s">
+      <c r="O32" s="7" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="33" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="7" t="s">
+    <row r="33" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="29" t="s">
+        <v>1621</v>
+      </c>
+      <c r="C33" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="D33" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="E33" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="F33" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="G33" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="G33" s="7">
+      <c r="H33" s="7">
         <v>1998</v>
       </c>
-      <c r="H33" s="7" t="s">
+      <c r="I33" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="I33" s="10">
+      <c r="J33" s="10">
         <v>471629847</v>
       </c>
-      <c r="J33" s="7" t="s">
+      <c r="K33" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="K33" s="7">
+      <c r="L33" s="7">
         <v>26</v>
       </c>
-      <c r="L33" s="8" t="s">
+      <c r="M33" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="M33" s="7" t="s">
+      <c r="N33" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N33" s="7" t="s">
+      <c r="O33" s="7" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="34" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="7">
+    <row r="34" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="10">
         <v>10713370</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="29" t="s">
+        <v>1577</v>
+      </c>
+      <c r="C34" s="8" t="s">
         <v>348</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="D34" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="E34" s="7" t="s">
         <v>351</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="F34" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="G34" s="7" t="s">
         <v>352</v>
       </c>
-      <c r="G34" s="7">
+      <c r="H34" s="7">
         <v>2008</v>
       </c>
-      <c r="H34" s="7" t="s">
+      <c r="I34" s="7" t="s">
         <v>353</v>
       </c>
-      <c r="I34" s="10" t="s">
+      <c r="J34" s="10" t="s">
         <v>350</v>
       </c>
-      <c r="K34" s="7">
+      <c r="L34" s="7">
         <v>25</v>
       </c>
-      <c r="L34" s="8" t="s">
+      <c r="M34" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="M34" s="7" t="s">
+      <c r="N34" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N34" s="9" t="s">
+      <c r="O34" s="9" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="35" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="7" t="s">
+    <row r="35" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="29" t="s">
+        <v>1579</v>
+      </c>
+      <c r="C35" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="D35" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="E35" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="F35" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="F35" s="7" t="s">
+      <c r="G35" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="G35" s="7">
+      <c r="H35" s="7">
         <v>1989</v>
       </c>
-      <c r="H35" s="7" t="s">
+      <c r="I35" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="I35" s="10">
+      <c r="J35" s="10">
         <v>139416420</v>
       </c>
-      <c r="J35" s="7" t="s">
+      <c r="K35" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="K35" s="7">
+      <c r="L35" s="7">
         <v>27</v>
       </c>
-      <c r="L35" s="8" t="s">
+      <c r="M35" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="M35" s="7" t="s">
+      <c r="N35" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N35" s="7" t="s">
+      <c r="O35" s="7" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="36" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="7">
+    <row r="36" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="23">
         <v>9071131</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="B36" s="29" t="s">
+        <v>1624</v>
+      </c>
+      <c r="C36" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="D36" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="E36" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="E36" s="7" t="s">
+      <c r="F36" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F36" s="7" t="s">
+      <c r="G36" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="G36" s="7">
+      <c r="H36" s="7">
         <v>1998</v>
       </c>
-      <c r="H36" s="7" t="s">
+      <c r="I36" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="I36" s="17">
+      <c r="J36" s="17">
         <v>201598817</v>
       </c>
-      <c r="J36" s="7" t="s">
+      <c r="K36" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="K36" s="7">
+      <c r="L36" s="7">
         <v>26</v>
       </c>
-      <c r="L36" s="8" t="s">
+      <c r="M36" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="M36" s="7" t="s">
+      <c r="N36" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N36" s="7" t="s">
+      <c r="O36" s="7" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="37" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="7">
+    <row r="37" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="10">
         <v>224864</v>
       </c>
-      <c r="B37" s="7" t="s">
+      <c r="B37" s="29" t="s">
+        <v>1578</v>
+      </c>
+      <c r="C37" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="D37" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="D37" s="7" t="s">
+      <c r="E37" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="E37" s="8" t="s">
+      <c r="F37" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="F37" s="7" t="s">
+      <c r="G37" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="G37" s="7">
+      <c r="H37" s="7">
         <v>1987</v>
       </c>
-      <c r="H37" s="7" t="s">
+      <c r="I37" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="I37" s="17">
+      <c r="J37" s="17">
         <v>70045801</v>
       </c>
-      <c r="J37" s="7" t="s">
+      <c r="K37" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="K37" s="7">
+      <c r="L37" s="7">
         <v>28</v>
       </c>
-      <c r="L37" s="8" t="s">
+      <c r="M37" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="M37" s="7" t="s">
+      <c r="N37" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N37" s="7" t="s">
+      <c r="O37" s="7" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="38" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="7" t="s">
+    <row r="38" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="B38" s="29" t="s">
+        <v>1580</v>
+      </c>
+      <c r="C38" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="D38" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="E38" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="E38" s="8" t="s">
+      <c r="F38" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="F38" s="7" t="s">
+      <c r="G38" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="G38" s="8" t="s">
+      <c r="H38" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="H38" s="7" t="s">
+      <c r="I38" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="I38" s="10">
+      <c r="J38" s="10">
         <v>70996946</v>
       </c>
-      <c r="J38" s="7" t="s">
+      <c r="K38" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="K38" s="7">
+      <c r="L38" s="7">
         <v>29</v>
       </c>
-      <c r="L38" s="8" t="s">
+      <c r="M38" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="M38" s="7" t="s">
+      <c r="N38" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N38" s="7" t="s">
+      <c r="O38" s="7" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="39" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="7" t="s">
+    <row r="39" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="B39" s="7" t="s">
+      <c r="B39" s="29" t="s">
+        <v>1581</v>
+      </c>
+      <c r="C39" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="D39" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="E39" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="E39" s="8" t="s">
+      <c r="F39" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="F39" s="7" t="s">
+      <c r="G39" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="G39" s="7" t="s">
+      <c r="H39" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="H39" s="7" t="s">
+      <c r="I39" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="I39" s="10">
+      <c r="J39" s="10">
         <v>72373385</v>
       </c>
-      <c r="J39" s="7" t="s">
+      <c r="K39" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="K39" s="7">
+      <c r="L39" s="7">
         <v>30</v>
       </c>
-      <c r="L39" s="8" t="s">
+      <c r="M39" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="M39" s="7" t="s">
+      <c r="N39" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N39" s="7" t="s">
+      <c r="O39" s="7" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="40" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="7" t="s">
+    <row r="40" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="29" t="s">
+        <v>1582</v>
+      </c>
+      <c r="C40" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="D40" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="E40" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="E40" s="8" t="s">
+      <c r="F40" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="F40" s="7" t="s">
+      <c r="G40" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="G40" s="7">
+      <c r="H40" s="7">
         <v>2001</v>
       </c>
-      <c r="H40" s="7" t="s">
+      <c r="I40" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="I40" s="17">
+      <c r="J40" s="17">
         <v>9775499569</v>
       </c>
-      <c r="J40" s="7" t="s">
+      <c r="K40" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="K40" s="7">
+      <c r="L40" s="7">
         <v>26</v>
       </c>
-      <c r="L40" s="8" t="s">
+      <c r="M40" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="M40" s="8" t="s">
+      <c r="N40" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="N40" s="9" t="s">
+      <c r="O40" s="9" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="41" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="7">
+    <row r="41" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="23">
         <v>13065685</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B41" s="29" t="s">
+        <v>1624</v>
+      </c>
+      <c r="C41" s="8" t="s">
         <v>343</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="D41" s="8" t="s">
         <v>344</v>
       </c>
-      <c r="D41" s="7" t="s">
+      <c r="E41" s="7" t="s">
         <v>346</v>
       </c>
-      <c r="E41" s="7" t="s">
+      <c r="F41" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F41" s="7" t="s">
+      <c r="G41" s="7" t="s">
         <v>341</v>
       </c>
-      <c r="G41" s="7">
+      <c r="H41" s="7">
         <v>2009</v>
       </c>
-      <c r="H41" s="7" t="s">
+      <c r="I41" s="7" t="s">
         <v>342</v>
       </c>
-      <c r="I41" s="18" t="s">
+      <c r="J41" s="18" t="s">
         <v>345</v>
       </c>
-      <c r="K41" s="7">
+      <c r="L41" s="7">
         <v>23</v>
       </c>
-      <c r="L41" s="8" t="s">
+      <c r="M41" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="M41" s="7" t="s">
+      <c r="N41" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="N41" s="9" t="s">
+      <c r="O41" s="9" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="42" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="2" t="s">
+    <row r="42" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="28" t="s">
+        <v>1591</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="D42" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="E42" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="E42" s="4" t="s">
+      <c r="F42" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="F42" s="2" t="s">
+      <c r="G42" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="G42" s="2">
+      <c r="H42" s="2">
         <v>2005</v>
       </c>
-      <c r="H42" s="2" t="s">
+      <c r="I42" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I42" s="6" t="s">
+      <c r="J42" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="J42" s="2" t="s">
+      <c r="K42" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="K42" s="2">
+      <c r="L42" s="2">
         <v>14</v>
       </c>
-      <c r="L42" s="2" t="s">
+      <c r="M42" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="M42" s="4" t="s">
+      <c r="N42" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="N42" s="2" t="s">
+      <c r="O42" s="2" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="43" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="2" t="s">
+    <row r="43" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="25" t="s">
         <v>255</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="28" t="s">
+        <v>1622</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="D43" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="D43" s="13" t="s">
+      <c r="E43" s="13" t="s">
         <v>261</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="F43" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F43" s="2" t="s">
+      <c r="G43" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="G43" s="2">
+      <c r="H43" s="2">
         <v>1993</v>
       </c>
-      <c r="H43" s="2" t="s">
+      <c r="I43" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="I43" s="4" t="s">
+      <c r="J43" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="J43" s="2" t="s">
+      <c r="K43" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="K43" s="2">
+      <c r="L43" s="2">
         <v>20</v>
       </c>
-      <c r="L43" s="2" t="s">
+      <c r="M43" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="M43" s="2" t="s">
+      <c r="N43" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N43" s="2" t="s">
+      <c r="O43" s="2" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="44" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="2" t="s">
+    <row r="44" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="28" t="s">
+        <v>1592</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="D44" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="E44" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="E44" s="4" t="s">
+      <c r="F44" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="F44" s="2" t="s">
+      <c r="G44" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="G44" s="2">
+      <c r="H44" s="2">
         <v>1998</v>
       </c>
-      <c r="H44" s="2" t="s">
+      <c r="I44" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="I44" s="2" t="s">
+      <c r="J44" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="J44" s="2" t="s">
+      <c r="K44" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="K44" s="2">
+      <c r="L44" s="2">
         <v>16</v>
       </c>
-      <c r="L44" s="2" t="s">
+      <c r="M44" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="M44" s="2" t="s">
+      <c r="N44" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N44" s="2" t="s">
+      <c r="O44" s="2" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="45" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="2" t="s">
+    <row r="45" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="25" t="s">
         <v>271</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" s="28" t="s">
+        <v>1623</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="D45" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="E45" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="F45" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="F45" s="2" t="s">
+      <c r="G45" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="G45" s="2">
+      <c r="H45" s="2">
         <v>1988</v>
       </c>
-      <c r="H45" s="2" t="s">
+      <c r="I45" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="I45" s="6" t="s">
+      <c r="J45" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="J45" s="2" t="s">
+      <c r="K45" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="K45" s="2">
+      <c r="L45" s="2">
         <v>17</v>
       </c>
-      <c r="L45" s="2" t="s">
+      <c r="M45" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="M45" s="2" t="s">
+      <c r="N45" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N45" s="2" t="s">
+      <c r="O45" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="46" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="2" t="s">
+    <row r="46" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="28" t="s">
+        <v>1593</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="D46" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="D46" s="2" t="s">
+      <c r="E46" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="E46" s="4" t="s">
+      <c r="F46" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="F46" s="2" t="s">
+      <c r="G46" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="G46" s="2">
+      <c r="H46" s="2">
         <v>2008</v>
       </c>
-      <c r="H46" s="2" t="s">
+      <c r="I46" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="I46" s="2">
+      <c r="J46" s="2">
         <v>9780132397285</v>
       </c>
-      <c r="J46" s="2" t="s">
+      <c r="K46" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="K46" s="2">
+      <c r="L46" s="2">
         <v>14</v>
       </c>
-      <c r="L46" s="2" t="s">
+      <c r="M46" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="M46" s="2" t="s">
+      <c r="N46" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N46" s="2" t="s">
+      <c r="O46" s="2" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="47" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="2" t="s">
+    <row r="47" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="3" t="s">
         <v>287</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="28" t="s">
+        <v>1594</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="D47" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="D47" s="2" t="s">
+      <c r="E47" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="E47" s="2" t="s">
+      <c r="F47" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="F47" s="2" t="s">
+      <c r="G47" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="G47" s="2">
+      <c r="H47" s="2">
         <v>1997</v>
       </c>
-      <c r="H47" s="2" t="s">
+      <c r="I47" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="I47" s="2">
+      <c r="J47" s="2">
         <v>134905253</v>
       </c>
-      <c r="J47" s="2" t="s">
+      <c r="K47" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="K47" s="2">
+      <c r="L47" s="2">
         <v>17</v>
       </c>
-      <c r="L47" s="2" t="s">
+      <c r="M47" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="M47" s="2" t="s">
+      <c r="N47" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N47" s="2" t="s">
+      <c r="O47" s="2" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="48" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="2" t="s">
+    <row r="48" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="28" t="s">
+        <v>1595</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="D48" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="E48" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="E48" s="2" t="s">
+      <c r="F48" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="F48" s="2" t="s">
+      <c r="G48" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="G48" s="4" t="s">
+      <c r="H48" s="4" t="s">
         <v>300</v>
       </c>
-      <c r="H48" s="2" t="s">
+      <c r="I48" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="I48" s="2">
+      <c r="J48" s="2">
         <v>9780538497817</v>
       </c>
-      <c r="J48" s="2" t="s">
+      <c r="K48" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="K48" s="2">
+      <c r="L48" s="2">
         <v>14</v>
       </c>
-      <c r="L48" s="2" t="s">
+      <c r="M48" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="M48" s="2" t="s">
+      <c r="N48" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N48" s="5" t="s">
+      <c r="O48" s="5" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="49" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="2" t="s">
+    <row r="49" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" s="28" t="s">
+        <v>1596</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="D49" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="D49" s="2" t="s">
+      <c r="E49" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="E49" s="4" t="s">
+      <c r="F49" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="F49" s="2" t="s">
+      <c r="G49" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="G49" s="2">
+      <c r="H49" s="2">
         <v>2004</v>
       </c>
-      <c r="H49" s="2" t="s">
+      <c r="I49" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I49" s="6" t="s">
+      <c r="J49" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="J49" s="2" t="s">
+      <c r="K49" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="K49" s="2">
+      <c r="L49" s="2">
         <v>14</v>
       </c>
-      <c r="L49" s="2" t="s">
+      <c r="M49" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="M49" s="2" t="s">
+      <c r="N49" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N49" s="2" t="s">
+      <c r="O49" s="2" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="50" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="2" t="s">
+    <row r="50" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="28" t="s">
+        <v>1597</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="D50" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="D50" s="2" t="s">
+      <c r="E50" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="E50" s="2" t="s">
+      <c r="F50" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="G50" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="G50" s="2">
+      <c r="H50" s="2">
         <v>2007</v>
       </c>
-      <c r="H50" s="2" t="s">
+      <c r="I50" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="I50" s="2">
+      <c r="J50" s="2">
         <v>9780199205226</v>
       </c>
-      <c r="J50" s="2" t="s">
+      <c r="K50" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="K50" s="2">
+      <c r="L50" s="2">
         <v>13</v>
       </c>
-      <c r="L50" s="2" t="s">
+      <c r="M50" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="M50" s="2" t="s">
+      <c r="N50" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N50" s="5" t="s">
+      <c r="O50" s="5" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="51" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="2" t="s">
+    <row r="51" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="28" t="s">
+        <v>1598</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="D51" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="D51" s="2" t="s">
+      <c r="E51" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="E51" s="4" t="s">
+      <c r="F51" s="4" t="s">
         <v>314</v>
       </c>
-      <c r="F51" s="2" t="s">
+      <c r="G51" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="G51" s="4" t="s">
+      <c r="H51" s="4" t="s">
         <v>317</v>
       </c>
-      <c r="H51" s="2" t="s">
+      <c r="I51" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="I51" s="2">
+      <c r="J51" s="2">
         <v>9780124059351</v>
       </c>
-      <c r="K51" s="2">
+      <c r="L51" s="2">
         <v>16</v>
       </c>
-      <c r="L51" s="2" t="s">
+      <c r="M51" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="M51" s="2" t="s">
+      <c r="N51" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N51" s="2" t="s">
+      <c r="O51" s="2" t="s">
         <v>318</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+  </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N2" r:id="rId1" xr:uid="{DE8EF3B1-71AA-4484-BCA9-E1FB86275EA2}"/>
-    <hyperlink ref="N3" r:id="rId2" xr:uid="{66EA466D-9A27-43BF-9228-C31DD48B05AB}"/>
-    <hyperlink ref="N4" r:id="rId3" xr:uid="{A6CF6CE5-F685-44A2-9B3D-33B11484695E}"/>
-    <hyperlink ref="N13" r:id="rId4" xr:uid="{8BDE62E3-78D2-4AE5-B32B-E3A0ECE41F81}"/>
-    <hyperlink ref="N14" r:id="rId5" xr:uid="{DD88F1B4-07F5-403C-AFFC-B1B83AF2C268}"/>
-    <hyperlink ref="N5" r:id="rId6" xr:uid="{118D1E05-349A-41F9-9AEB-90095200471C}"/>
-    <hyperlink ref="N40" r:id="rId7" xr:uid="{939D4173-5F07-48EB-A943-C0F68227C9D2}"/>
-    <hyperlink ref="N48" r:id="rId8" xr:uid="{DE815DD5-592E-4901-B2BE-F27CF4EE33EE}"/>
-    <hyperlink ref="N50" r:id="rId9" xr:uid="{86A2D858-A150-45C6-AFF2-81E4A169F1AA}"/>
-    <hyperlink ref="N26" r:id="rId10" xr:uid="{3CA31FF9-42C2-430E-A1A3-88FC1FDB06EF}"/>
-    <hyperlink ref="N29" r:id="rId11" xr:uid="{6C20E9FB-A615-44B6-9CD3-E6358AAE75E8}"/>
-    <hyperlink ref="N41" r:id="rId12" xr:uid="{E83B8283-F688-46E3-81C5-6EEA42717D07}"/>
-    <hyperlink ref="N34" r:id="rId13" xr:uid="{3C1A532F-A454-44EB-84B7-5A9D13E29979}"/>
-    <hyperlink ref="N6" r:id="rId14" xr:uid="{B9E35097-036D-45B4-ACA2-07F25FC924F9}"/>
-    <hyperlink ref="N7" r:id="rId15" xr:uid="{53EF9833-F58D-4EE3-A2AB-B249CF7DBE27}"/>
-    <hyperlink ref="N9" r:id="rId16" xr:uid="{82B0C102-B859-4C2B-9543-F83A138E7438}"/>
-    <hyperlink ref="N12" r:id="rId17" xr:uid="{533DDA2D-DCED-41B2-B65E-09B69B0BD310}"/>
-    <hyperlink ref="N15" r:id="rId18" xr:uid="{2D2E08B6-B3DE-4470-8FDB-3ED9A06011EB}"/>
-    <hyperlink ref="N18" r:id="rId19" xr:uid="{ABAF1F42-02B7-4323-836E-6DE114EB668F}"/>
-    <hyperlink ref="N19" r:id="rId20" xr:uid="{286CCA41-F868-4F40-9F8A-2404DF11D1CB}"/>
-    <hyperlink ref="N20" r:id="rId21" xr:uid="{C31C3FE9-494F-4EF8-A3EA-2830581171EF}"/>
+    <hyperlink ref="O2" r:id="rId1" xr:uid="{DE8EF3B1-71AA-4484-BCA9-E1FB86275EA2}"/>
+    <hyperlink ref="O3" r:id="rId2" xr:uid="{66EA466D-9A27-43BF-9228-C31DD48B05AB}"/>
+    <hyperlink ref="O4" r:id="rId3" xr:uid="{A6CF6CE5-F685-44A2-9B3D-33B11484695E}"/>
+    <hyperlink ref="O13" r:id="rId4" xr:uid="{8BDE62E3-78D2-4AE5-B32B-E3A0ECE41F81}"/>
+    <hyperlink ref="O14" r:id="rId5" xr:uid="{DD88F1B4-07F5-403C-AFFC-B1B83AF2C268}"/>
+    <hyperlink ref="O5" r:id="rId6" xr:uid="{118D1E05-349A-41F9-9AEB-90095200471C}"/>
+    <hyperlink ref="O40" r:id="rId7" xr:uid="{939D4173-5F07-48EB-A943-C0F68227C9D2}"/>
+    <hyperlink ref="O48" r:id="rId8" xr:uid="{DE815DD5-592E-4901-B2BE-F27CF4EE33EE}"/>
+    <hyperlink ref="O50" r:id="rId9" xr:uid="{86A2D858-A150-45C6-AFF2-81E4A169F1AA}"/>
+    <hyperlink ref="O26" r:id="rId10" xr:uid="{3CA31FF9-42C2-430E-A1A3-88FC1FDB06EF}"/>
+    <hyperlink ref="O29" r:id="rId11" xr:uid="{6C20E9FB-A615-44B6-9CD3-E6358AAE75E8}"/>
+    <hyperlink ref="O41" r:id="rId12" xr:uid="{E83B8283-F688-46E3-81C5-6EEA42717D07}"/>
+    <hyperlink ref="O34" r:id="rId13" xr:uid="{3C1A532F-A454-44EB-84B7-5A9D13E29979}"/>
+    <hyperlink ref="O6" r:id="rId14" xr:uid="{B9E35097-036D-45B4-ACA2-07F25FC924F9}"/>
+    <hyperlink ref="O7" r:id="rId15" xr:uid="{53EF9833-F58D-4EE3-A2AB-B249CF7DBE27}"/>
+    <hyperlink ref="O9" r:id="rId16" xr:uid="{82B0C102-B859-4C2B-9543-F83A138E7438}"/>
+    <hyperlink ref="O12" r:id="rId17" xr:uid="{533DDA2D-DCED-41B2-B65E-09B69B0BD310}"/>
+    <hyperlink ref="O15" r:id="rId18" xr:uid="{2D2E08B6-B3DE-4470-8FDB-3ED9A06011EB}"/>
+    <hyperlink ref="O18" r:id="rId19" xr:uid="{ABAF1F42-02B7-4323-836E-6DE114EB668F}"/>
+    <hyperlink ref="O19" r:id="rId20" xr:uid="{286CCA41-F868-4F40-9F8A-2404DF11D1CB}"/>
+    <hyperlink ref="O20" r:id="rId21" xr:uid="{C31C3FE9-494F-4EF8-A3EA-2830581171EF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId22"/>

</xml_diff>